<commit_message>
Add 161 converted CDS test cases in new Steps-sheet format
Auto-converted from Katalon SQLite Excel files in InputFiles/CDS/.
Each TC has Steps sheet: header row, config row, then steps —
dismiss_popup, nav, filter dropdowns+checkboxes, read_stat_bar,
multi_function for ParticipantsTab/SamplesTab/FilesTab.

Filters parsed from old SQL WHERE clause and mapped to new
Filter column key=value. 17 filter types supported:
phs, gender, sex, file_type, strategy, tumor_status, sample_type,
platform, instrument_model, library_strategy, library_source,
library_layout, library_selection, reference_genome,
primary_diagnosis, study_data_types, image_modality.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TestCases/TC01_CDS_phs001437_Sex-Unknown_ExperimentalStrategy-RNASeq.xlsx
+++ b/TestCases/TC01_CDS_phs001437_Sex-Unknown_ExperimentalStrategy-RNASeq.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K14"/>
+  <dimension ref="A1:K15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -455,7 +455,7 @@
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="22" customWidth="1" min="6" max="6"/>
     <col width="15" customWidth="1" min="7" max="7"/>
-    <col width="55" customWidth="1" min="8" max="8"/>
+    <col width="60" customWidth="1" min="8" max="8"/>
     <col width="18" customWidth="1" min="9" max="9"/>
     <col width="20" customWidth="1" min="10" max="10"/>
     <col width="35" customWidth="1" min="11" max="11"/>
@@ -542,6 +542,10 @@
           <t>dismiss_popup</t>
         </is>
       </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
           <t>Dismiss warning popup</t>
@@ -567,6 +571,8 @@
           <t>CDS_Data-Btn</t>
         </is>
       </c>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr">
         <is>
           <t>Click Data nav button</t>
@@ -589,12 +595,14 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Filter/StudyFacet/PHS_Accession/PHS_Accession_Ddn</t>
-        </is>
-      </c>
+          <t>Data_page/Filter/StudyFacet/PHS_Accession/PHS_Accession_Ddn</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Expand PHS Accession</t>
+          <t>Expand phs filter</t>
         </is>
       </c>
     </row>
@@ -614,9 +622,10 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Filter/StudyFacet/PHS_Accession/phs001437_Chkbx</t>
-        </is>
-      </c>
+          <t>Data_page/Filter/StudyFacet/PHS_Accession/phs001437_Chkbx</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr"/>
       <c r="J6" s="3" t="inlineStr">
         <is>
           <t>phs=phs001437</t>
@@ -644,12 +653,14 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Filter/DemographicsFacet/Sex/Sex-Ddn</t>
-        </is>
-      </c>
+          <t>Data_page/Filter/DemographicsFacet/Gender/Gender-Ddn</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Expand Sex filter</t>
+          <t>Expand gender filter</t>
         </is>
       </c>
     </row>
@@ -669,12 +680,13 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Filter/DemographicsFacet/Sex/Unknown-Chkbx</t>
-        </is>
-      </c>
+          <t>Data_page/Filter/DemographicsFacet/Gender/Unknown-Chkbx</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr"/>
       <c r="J8" s="3" t="inlineStr">
         <is>
-          <t>sex=Unknown</t>
+          <t>gender=Unknown</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -699,12 +711,14 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Filter/StudyFacet/ExperimentalStrategy/ExperimentalStrategy_Ddn</t>
-        </is>
-      </c>
+          <t>Data_page/Filter/StudyFacet/ExperimentalStrategy/ExperimentalStrategy_Ddn</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Expand Experimental Strategy</t>
+          <t>Expand strategy filter</t>
         </is>
       </c>
     </row>
@@ -724,9 +738,10 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Filter/StudyFacet/ExperimentalStrategy/RNASeq-Chkbx</t>
-        </is>
-      </c>
+          <t>Data_page/Filter/StudyFacet/ExperimentalStrategy/RNA-Seq-Chkbx</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr"/>
       <c r="J10" s="3" t="inlineStr">
         <is>
           <t>strategy=RNA-Seq</t>
@@ -744,17 +759,28 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>read_stat_bar</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>CDS</t>
+          <t>js_click_and_wait</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Data_page</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Data_page/Filter/StudyFacet/ExperimentalStrategy/WXS-Chkbx</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" s="3" t="inlineStr">
+        <is>
+          <t>strategy=WXS</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>Read stat bar counts</t>
+          <t>Select WXS</t>
         </is>
       </c>
     </row>
@@ -764,17 +790,20 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>multi_function</t>
-        </is>
-      </c>
+          <t>read_stat_bar</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr">
         <is>
-          <t>ParticipantsTab</t>
-        </is>
-      </c>
+          <t>CDS</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr">
         <is>
-          <t>Compare Participants</t>
+          <t>Read stat bar counts</t>
         </is>
       </c>
     </row>
@@ -787,14 +816,17 @@
           <t>multi_function</t>
         </is>
       </c>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr">
         <is>
-          <t>SamplesTab</t>
-        </is>
-      </c>
+          <t>ParticipantsTab</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr">
         <is>
-          <t>Compare Samples</t>
+          <t>Compare ParticipantsTab</t>
         </is>
       </c>
     </row>
@@ -807,14 +839,40 @@
           <t>multi_function</t>
         </is>
       </c>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr">
         <is>
+          <t>SamplesTab</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>Compare SamplesTab</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>13</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>multi_function</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr">
+        <is>
           <t>FilesTab</t>
         </is>
       </c>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t>Compare Files</t>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>Compare FilesTab</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: resolve suite runner issues — Gender→Sex, stale DOM, obj key doubling
- run_suite.py: add --limit flag to cap number of TCs run
- test_runner.py: strip leading page_name/ from obj_name to prevent
  doubled key (CDS/Data_page/Data_page/Filter/...)
- test_runner.py: add _ensure_facet_expanded() — auto-expands collapsed
  filter sections (e.g. Demographics) before clicking a child element
- test_runner.py: add _FACET_EXPANDERS dict for CDS DemographicsFacet
- actions.py: click_and_wait now waits for networkidle before locating,
  uses JS scrollIntoView to avoid "not attached to DOM" on React re-renders
- TestCases: fix 45 TCs that used Gender→Sex (QA env only has Sex facet)
- TestCases: fix 10 TCs that used RNA-Seq-Chkbx / Targeted-Capture-Chkbx
  → RNASeq-Chkbx / TargetedCapture-Chkbx to match Object Repo key names

Result: 3/3 suite TCs now PASS (was 3/3 ERROR)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TestCases/TC01_CDS_phs001437_Sex-Unknown_ExperimentalStrategy-RNASeq.xlsx
+++ b/TestCases/TC01_CDS_phs001437_Sex-Unknown_ExperimentalStrategy-RNASeq.xlsx
@@ -542,10 +542,6 @@
           <t>dismiss_popup</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
           <t>Dismiss warning popup</t>
@@ -571,8 +567,6 @@
           <t>CDS_Data-Btn</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr">
         <is>
           <t>Click Data nav button</t>
@@ -598,8 +592,6 @@
           <t>Data_page/Filter/StudyFacet/PHS_Accession/PHS_Accession_Ddn</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr">
         <is>
           <t>Expand phs filter</t>
@@ -625,7 +617,6 @@
           <t>Data_page/Filter/StudyFacet/PHS_Accession/phs001437_Chkbx</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr"/>
       <c r="J6" s="3" t="inlineStr">
         <is>
           <t>phs=phs001437</t>
@@ -653,11 +644,9 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Data_page/Filter/DemographicsFacet/Gender/Gender-Ddn</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
+          <t>Data_page/Filter/DemographicsFacet/Sex/Sex-Ddn</t>
+        </is>
+      </c>
       <c r="K7" t="inlineStr">
         <is>
           <t>Expand gender filter</t>
@@ -680,13 +669,12 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Data_page/Filter/DemographicsFacet/Gender/Unknown-Chkbx</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr"/>
+          <t>Data_page/Filter/DemographicsFacet/Sex/Unknown-Chkbx</t>
+        </is>
+      </c>
       <c r="J8" s="3" t="inlineStr">
         <is>
-          <t>gender=Unknown</t>
+          <t>sex=Unknown</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -714,8 +702,6 @@
           <t>Data_page/Filter/StudyFacet/ExperimentalStrategy/ExperimentalStrategy_Ddn</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr">
         <is>
           <t>Expand strategy filter</t>
@@ -738,10 +724,9 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Data_page/Filter/StudyFacet/ExperimentalStrategy/RNA-Seq-Chkbx</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr"/>
+          <t>Data_page/Filter/StudyFacet/ExperimentalStrategy/RNASeq-Chkbx</t>
+        </is>
+      </c>
       <c r="J10" s="3" t="inlineStr">
         <is>
           <t>strategy=RNA-Seq</t>
@@ -772,7 +757,6 @@
           <t>Data_page/Filter/StudyFacet/ExperimentalStrategy/WXS-Chkbx</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr"/>
       <c r="J11" s="3" t="inlineStr">
         <is>
           <t>strategy=WXS</t>
@@ -793,14 +777,11 @@
           <t>read_stat_bar</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr">
         <is>
           <t>CDS</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr">
         <is>
           <t>Read stat bar counts</t>
@@ -816,14 +797,11 @@
           <t>multi_function</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr">
         <is>
           <t>ParticipantsTab</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr">
         <is>
           <t>Compare ParticipantsTab</t>
@@ -839,14 +817,11 @@
           <t>multi_function</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr">
         <is>
           <t>SamplesTab</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr">
         <is>
           <t>Compare SamplesTab</t>
@@ -862,14 +837,11 @@
           <t>multi_function</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr">
         <is>
           <t>FilesTab</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr">
         <is>
           <t>Compare FilesTab</t>

</xml_diff>